<commit_message>
Train_results_R2: add commonsense, rollback follow-up and cost rows
Adds the commonsense errors (start -> end) row, the rollback follow-up
rows (queries never accepted again, repeated rejected candidates) and
the rollback cost rows (tokens, time, discarded commonsense fixes),
computed from the run's own records. Rates use up to 2 decimals and the
sheet now carries the title row, borders and summary like Results.xlsx.
Also runs the analyzer in UTF-8 mode so the notebook works on Windows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/train_result_analysis/Train_results_R2.xlsx
+++ b/train_result_analysis/Train_results_R2.xlsx
@@ -37,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +45,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -425,142 +440,238 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>R2 training result</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Queries</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" s="3" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Repair attempts</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B4" s="3" t="n">
         <v>332</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Personal repair attempts</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B5" s="3" t="n">
         <v>141</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Commonsense repair attempts</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" s="3" t="n">
         <v>191</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Confirmed unchanged attempts</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>235 (70.78%)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Personal constraint fixes</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" s="3" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Personal regressions</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Harmful candidates blocked (rejected)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>25 / 332 (7.5%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>25 / 332 (7.53%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Rejected: fixed target but caused a protected regression</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>0 / 332 (0.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>0 / 332 (0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Rejected and loop continued</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>20 / 332 (6.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>20 / 332 (6.02%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Rejected candidate differed from accepted plan</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>25 / 25 (100.0%)</t>
-        </is>
-      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>25 / 25 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Commonsense errors (start → end)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>304 → 271 (−10.9%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Queries never accepted again after first rejection</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>5 / 5 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Rejected candidates identical to an earlier rejected one</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>6 / 25 (24%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Tokens spent on rejected candidates</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>0.89M / 5.63M (15.72%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Time spent on rejected candidates</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>803 s / 6,261 s (12.82%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Commonsense fixes discarded by rejections</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Summary</t>
+          </r>
+          <r>
+            <t>: R2 rejected 25 harmful candidates (7.5% of attempts), preventing any protected-constraint regression. This is consistent with its design. The cost is caution: only 2 personal fixes and ~71% of attempts unchanged.</t>
+          </r>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A22:B22"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Train_results_R2: remove the summary from notebook and xlsx
Keep the teammate's added rows (commonsense start->end, rejection follow-up,
rollback cost) but drop the summary sentence/block so R2 matches R0/R3 (table
only, no summary).
</commit_message>
<xml_diff>
--- a/train_result_analysis/Train_results_R2.xlsx
+++ b/train_result_analysis/Train_results_R2.xlsx
@@ -55,7 +55,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -63,9 +63,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -432,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -652,26 +649,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>Summary</t>
-          </r>
-          <r>
-            <t>: R2 rejected 25 harmful candidates (7.5% of attempts), preventing any protected-constraint regression. This is consistent with its design. The cost is caution: only 2 personal fixes and ~71% of attempts unchanged.</t>
-          </r>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A22:B22"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated with r0's format
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/train_result_analysis/Train_results_R2.xlsx
+++ b/train_result_analysis/Train_results_R2.xlsx
@@ -37,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,25 +45,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,224 +424,458 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>R2</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>R2 TRAIN result</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>R2 training result</t>
-        </is>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Queries evaluated</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Queries</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>60</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total repair attempts</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>332</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Repair attempts</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>332</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Personal-constraint repair attempts</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>141</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Personal repair attempts</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>141</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Commonsense repair attempts</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>191</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Commonsense repair attempts</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>191</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Attempts that left the plan unchanged</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>235 (70.78%)</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed unchanged attempts</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>235 (70.78%)</t>
-        </is>
+          <t>Personal constraints fixed (across attempts)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Personal constraint fixes</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>2</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Personal constraints newly broken (across attempts)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Personal regressions</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Queries improved</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>4/60 (6.7%)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Queries unchanged</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>55/60 (91.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Queries worsened</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1/60 (1.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Net personal constraints gained</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Commonsense errors (start → end)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>304 → 271 (−10.9%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Attempts with confirmed no change</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>214/332 (64.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Changed and fixed ≥1 without regression</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1/332 (0.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Changed and introduced a regression</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>18/332 (5.4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rollback (R2)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Harmful candidates blocked (rejected)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>25 / 332 (7.53%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>25 / 332 (7.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rollback (R2)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Rejected: fixed target but caused a protected regression</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>0 / 332 (0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0 / 332 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rollback (R2)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Rejected and loop continued</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>20 / 332 (6.02%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>20 / 332 (6.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rollback (R2)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Rejected candidate differed from accepted plan</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>25 / 25 (100%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Commonsense errors (start → end)</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>304 → 271 (−10.9%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>25 / 25 (100.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rollback (R2)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Queries never accepted again after first rejection</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>5 / 5 (100%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>5 / 5 (100.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rollback (R2)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Rejected candidates identical to an earlier rejected one</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6 / 25 (24%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>6 / 25 (24.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rollback cost (R2)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Tokens spent on rejected candidates</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>0.89M / 5.63M (15.72%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0.89M / 5.63M (15.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rollback cost (R2)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Time spent on rejected candidates</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>803 s / 6,261 s (12.82%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>803 s / 6,261 s (12.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Rollback cost (R2)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Commonsense fixes discarded by rejections</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="C26" s="4" t="n">
         <v>64</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Average tokens per query</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>99257</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Average repair time per query</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>109.4 s</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>